<commit_message>
Fill Cottage Bakery demo with US prices; add HOW-TO-USE guide
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cottage-bakery-spreadsheet/Cottage_Bakery_v4_ENHANCED.xlsx
+++ b/cottage-bakery-spreadsheet/Cottage_Bakery_v4_ENHANCED.xlsx
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>My Cottage Bakery</t>
+          <t>Rose &amp; Rye Cottage Bakery</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Your Name</t>
+          <t>Jane Miller</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Can auto from Overhead tab or manual</t>
+          <t>Manual %, or copy Overhead Expenses!B28 for auto</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>45658</v>
+        <v>46023</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
@@ -1991,11 +1991,11 @@
         </is>
       </c>
       <c r="B2" s="63" t="n">
-        <v>45855</v>
+        <v>46254</v>
       </c>
       <c r="C2" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D2" s="64" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B3" s="63" t="n">
-        <v>45840</v>
+        <v>46248</v>
       </c>
       <c r="C3" s="64" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="B4" s="63" t="n">
-        <v>45855</v>
+        <v>46260</v>
       </c>
       <c r="C4" s="64" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="B5" s="63" t="n">
-        <v>45847</v>
+        <v>46244</v>
       </c>
       <c r="C5" s="64" t="inlineStr">
         <is>
@@ -2215,11 +2215,11 @@
         </is>
       </c>
       <c r="B6" s="63" t="n">
-        <v>45850</v>
+        <v>46251</v>
       </c>
       <c r="C6" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D6" s="64" t="inlineStr">
@@ -2271,11 +2271,11 @@
         </is>
       </c>
       <c r="B7" s="63" t="n">
-        <v>45839</v>
+        <v>46260</v>
       </c>
       <c r="C7" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B8" s="63" t="n">
-        <v>45840</v>
+        <v>46259</v>
       </c>
       <c r="C8" s="64" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="B9" s="63" t="n">
-        <v>45853</v>
+        <v>46260</v>
       </c>
       <c r="C9" s="64" t="inlineStr">
         <is>
@@ -2439,11 +2439,11 @@
         </is>
       </c>
       <c r="B10" s="63" t="n">
-        <v>45852</v>
+        <v>46252</v>
       </c>
       <c r="C10" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D10" s="64" t="inlineStr">
@@ -2495,11 +2495,11 @@
         </is>
       </c>
       <c r="B11" s="63" t="n">
-        <v>45842</v>
+        <v>46253</v>
       </c>
       <c r="C11" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D11" s="64" t="inlineStr">
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="B12" s="63" t="n">
-        <v>45858</v>
+        <v>46243</v>
       </c>
       <c r="C12" s="64" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="B13" s="63" t="n">
-        <v>45855</v>
+        <v>46261</v>
       </c>
       <c r="C13" s="64" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
         </is>
       </c>
       <c r="B14" s="63" t="n">
-        <v>45852</v>
+        <v>46255</v>
       </c>
       <c r="C14" s="64" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="B15" s="63" t="n">
-        <v>45850</v>
+        <v>46252</v>
       </c>
       <c r="C15" s="64" t="inlineStr">
         <is>
@@ -2775,11 +2775,11 @@
         </is>
       </c>
       <c r="B16" s="63" t="n">
-        <v>45840</v>
+        <v>46262</v>
       </c>
       <c r="C16" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D16" s="64" t="inlineStr">
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="B17" s="63" t="n">
-        <v>45851</v>
+        <v>46253</v>
       </c>
       <c r="C17" s="64" t="inlineStr">
         <is>
@@ -2887,11 +2887,11 @@
         </is>
       </c>
       <c r="B18" s="63" t="n">
-        <v>45844</v>
+        <v>46261</v>
       </c>
       <c r="C18" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D18" s="64" t="inlineStr">
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="B19" s="63" t="n">
-        <v>45843</v>
+        <v>46260</v>
       </c>
       <c r="C19" s="64" t="inlineStr">
         <is>
@@ -2999,11 +2999,11 @@
         </is>
       </c>
       <c r="B20" s="63" t="n">
-        <v>45855</v>
+        <v>46235</v>
       </c>
       <c r="C20" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D20" s="64" t="inlineStr">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="B21" s="63" t="n">
-        <v>45852</v>
+        <v>46252</v>
       </c>
       <c r="C21" s="64" t="inlineStr">
         <is>
@@ -3285,11 +3285,11 @@
         <v>1</v>
       </c>
       <c r="B2" s="53" t="n">
-        <v>45840</v>
+        <v>46236</v>
       </c>
       <c r="C2" s="31" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D2" s="31" t="inlineStr">
@@ -3321,7 +3321,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="53" t="n">
-        <v>45841</v>
+        <v>46237</v>
       </c>
       <c r="C3" s="31" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="53" t="n">
-        <v>45842</v>
+        <v>46238</v>
       </c>
       <c r="C4" s="31" t="inlineStr">
         <is>
@@ -3393,11 +3393,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="53" t="n">
-        <v>45843</v>
+        <v>46239</v>
       </c>
       <c r="C5" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D5" s="31" t="inlineStr">
@@ -3429,11 +3429,11 @@
         <v>5</v>
       </c>
       <c r="B6" s="53" t="n">
-        <v>45844</v>
+        <v>46240</v>
       </c>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D6" s="31" t="inlineStr">
@@ -3465,7 +3465,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="53" t="n">
-        <v>45845</v>
+        <v>46241</v>
       </c>
       <c r="C7" s="31" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="53" t="n">
-        <v>45846</v>
+        <v>46242</v>
       </c>
       <c r="C8" s="31" t="inlineStr">
         <is>
@@ -3537,11 +3537,11 @@
         <v>8</v>
       </c>
       <c r="B9" s="53" t="n">
-        <v>45847</v>
+        <v>46243</v>
       </c>
       <c r="C9" s="31" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D9" s="31" t="inlineStr">
@@ -3573,11 +3573,11 @@
         <v>9</v>
       </c>
       <c r="B10" s="53" t="n">
-        <v>45848</v>
+        <v>46244</v>
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D10" s="31" t="inlineStr">
@@ -3609,7 +3609,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="53" t="n">
-        <v>45849</v>
+        <v>46245</v>
       </c>
       <c r="C11" s="31" t="inlineStr">
         <is>
@@ -3837,7 +3837,7 @@
     </row>
     <row r="2">
       <c r="A2" s="53" t="n">
-        <v>45840</v>
+        <v>46236</v>
       </c>
       <c r="B2" s="31" t="inlineStr">
         <is>
@@ -3865,7 +3865,7 @@
     </row>
     <row r="3">
       <c r="A3" s="53" t="n">
-        <v>45841</v>
+        <v>46237</v>
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
     </row>
     <row r="4">
       <c r="A4" s="53" t="n">
-        <v>45842</v>
+        <v>46238</v>
       </c>
       <c r="B4" s="31" t="inlineStr">
         <is>
@@ -3921,7 +3921,7 @@
     </row>
     <row r="5">
       <c r="A5" s="53" t="n">
-        <v>45843</v>
+        <v>46239</v>
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
@@ -3949,7 +3949,7 @@
     </row>
     <row r="6">
       <c r="A6" s="53" t="n">
-        <v>45844</v>
+        <v>46240</v>
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
@@ -3977,7 +3977,7 @@
     </row>
     <row r="7">
       <c r="A7" s="53" t="n">
-        <v>45845</v>
+        <v>46241</v>
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
@@ -4005,7 +4005,7 @@
     </row>
     <row r="8">
       <c r="A8" s="53" t="n">
-        <v>45846</v>
+        <v>46242</v>
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
     </row>
     <row r="9">
       <c r="A9" s="53" t="n">
-        <v>45847</v>
+        <v>46243</v>
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
@@ -4061,7 +4061,7 @@
     </row>
     <row r="10">
       <c r="A10" s="53" t="n">
-        <v>45848</v>
+        <v>46244</v>
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
     </row>
     <row r="11">
       <c r="A11" s="53" t="n">
-        <v>45849</v>
+        <v>46245</v>
       </c>
       <c r="B11" s="31" t="inlineStr">
         <is>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B2" s="31" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D2">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D3">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B4" s="31" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D4">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D6">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D8">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D9">
@@ -5655,10 +5655,10 @@
         </is>
       </c>
       <c r="E2" s="7" t="n">
-        <v>5000</v>
+        <v>2268</v>
       </c>
       <c r="F2" s="20" t="n">
-        <v>6.5</v>
+        <v>6.99</v>
       </c>
       <c r="G2" s="21">
         <f>IF(E2=0,0,F2/E2)</f>
@@ -5680,17 +5680,17 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>Bob's Mill</t>
+          <t>King Arthur</t>
         </is>
       </c>
       <c r="M2" s="22" t="n">
-        <v>45839</v>
+        <v>46235</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>5000</v>
+        <v>4536</v>
       </c>
       <c r="O2" s="22" t="n">
-        <v>46023</v>
+        <v>46600</v>
       </c>
       <c r="P2" s="7" t="inlineStr">
         <is>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="Q2" s="7" t="inlineStr">
         <is>
-          <t>Organic</t>
+          <t>5 lb bag</t>
         </is>
       </c>
       <c r="R2" s="7">
@@ -5713,12 +5713,12 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Sugar</t>
+          <t>All-Purpose Flour</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Sugar</t>
+          <t>Flour</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -5727,20 +5727,20 @@
         </is>
       </c>
       <c r="E3" s="8" t="n">
-        <v>2000</v>
+        <v>2268</v>
       </c>
       <c r="F3" s="23" t="n">
-        <v>3.2</v>
+        <v>4.99</v>
       </c>
       <c r="G3" s="24">
         <f>IF(E3=0,0,F3/E3)</f>
         <v/>
       </c>
       <c r="H3" s="8" t="n">
-        <v>800</v>
+        <v>3000</v>
       </c>
       <c r="I3" s="8" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="J3" s="23">
         <f>H3*G3</f>
@@ -5752,24 +5752,28 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Costco</t>
+          <t>Gold Medal</t>
         </is>
       </c>
       <c r="M3" s="25" t="n">
-        <v>45848</v>
+        <v>46239</v>
       </c>
       <c r="N3" s="8" t="n">
-        <v>2000</v>
+        <v>4536</v>
       </c>
       <c r="O3" s="25" t="n">
-        <v>46204</v>
+        <v>46419</v>
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Pantry A</t>
         </is>
       </c>
-      <c r="Q3" s="8" t="inlineStr"/>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>5 lb bag</t>
+        </is>
+      </c>
       <c r="R3" s="8">
         <f>IFERROR(VLOOKUP(D3,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
@@ -5781,12 +5785,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Sugar</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Sugar</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -5795,17 +5799,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>1000</v>
+        <v>1814</v>
       </c>
       <c r="F4" s="20" t="n">
-        <v>8.99</v>
+        <v>3.29</v>
       </c>
       <c r="G4" s="21">
         <f>IF(E4=0,0,F4/E4)</f>
         <v/>
       </c>
       <c r="H4" s="7" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="I4" s="7" t="n">
         <v>500</v>
@@ -5820,26 +5824,26 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="M4" s="22" t="n">
-        <v>45853</v>
+        <v>46242</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>1000</v>
+        <v>1814</v>
       </c>
       <c r="O4" s="22" t="n">
-        <v>45870</v>
+        <v>46600</v>
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>Fridge</t>
+          <t>Pantry A</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>European</t>
+          <t>4 lb bag</t>
         </is>
       </c>
       <c r="R4" s="7">
@@ -5853,34 +5857,34 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Eggs</t>
+          <t>Brown Sugar</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Sugar</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E5" s="8" t="n">
-        <v>12</v>
+        <v>907</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>5.5</v>
+        <v>2.79</v>
       </c>
       <c r="G5" s="24">
         <f>IF(E5=0,0,F5/E5)</f>
         <v/>
       </c>
       <c r="H5" s="8" t="n">
-        <v>18</v>
+        <v>400</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>12</v>
+        <v>250</v>
       </c>
       <c r="J5" s="23">
         <f>H5*G5</f>
@@ -5892,26 +5896,26 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>Farm</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="M5" s="25" t="n">
-        <v>45856</v>
+        <v>46242</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>24</v>
+        <v>907</v>
       </c>
       <c r="O5" s="25" t="n">
-        <v>45874</v>
+        <v>46600</v>
       </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
-          <t>Fridge</t>
+          <t>Pantry A</t>
         </is>
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Free range</t>
+          <t>2 lb bag</t>
         </is>
       </c>
       <c r="R5" s="8">
@@ -5925,34 +5929,34 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Vanilla Extract</t>
+          <t>Butter</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Flavoring</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>200</v>
+        <v>454</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>12</v>
+        <v>4.49</v>
       </c>
       <c r="G6" s="21">
         <f>IF(E6=0,0,F6/E6)</f>
         <v/>
       </c>
       <c r="H6" s="7" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="J6" s="20">
         <f>H6*G6</f>
@@ -5964,26 +5968,26 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>Nielsen</t>
+          <t>Land O'Lakes</t>
         </is>
       </c>
       <c r="M6" s="22" t="n">
-        <v>45828</v>
+        <v>46254</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>200</v>
+        <v>908</v>
       </c>
       <c r="O6" s="22" t="n">
-        <v>46539</v>
+        <v>46296</v>
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>Rack</t>
+          <t>Fridge</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>Pure</t>
+          <t>1 lb, unsalted</t>
         </is>
       </c>
       <c r="R6" s="7">
@@ -5997,34 +6001,34 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Chocolate Chips</t>
+          <t>Eggs</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Chocolate</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1500</v>
+        <v>12</v>
       </c>
       <c r="F7" s="23" t="n">
-        <v>9.75</v>
+        <v>3.99</v>
       </c>
       <c r="G7" s="24">
         <f>IF(E7=0,0,F7/E7)</f>
         <v/>
       </c>
       <c r="H7" s="8" t="n">
-        <v>1200</v>
+        <v>18</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>400</v>
+        <v>12</v>
       </c>
       <c r="J7" s="23">
         <f>H7*G7</f>
@@ -6036,26 +6040,26 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>Ghirardelli</t>
+          <t>Eggland's Best</t>
         </is>
       </c>
       <c r="M7" s="25" t="n">
-        <v>45843</v>
+        <v>46256</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>1500</v>
+        <v>24</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>46208</v>
+        <v>46285</v>
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Pantry B</t>
+          <t>Fridge</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Semi</t>
+          <t>Large, cage-free</t>
         </is>
       </c>
       <c r="R7" s="8">
@@ -6069,34 +6073,34 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Cream Cheese</t>
+          <t>Vanilla Extract</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Flavoring</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>500</v>
+        <v>59</v>
       </c>
       <c r="F8" s="20" t="n">
-        <v>4.25</v>
+        <v>12.99</v>
       </c>
       <c r="G8" s="21">
         <f>IF(E8=0,0,F8/E8)</f>
         <v/>
       </c>
       <c r="H8" s="7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="J8" s="20">
         <f>H8*G8</f>
@@ -6108,26 +6112,26 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Nielsen-Massey</t>
         </is>
       </c>
       <c r="M8" s="22" t="n">
-        <v>45850</v>
+        <v>46213</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>1000</v>
+        <v>118</v>
       </c>
       <c r="O8" s="22" t="n">
-        <v>45866</v>
+        <v>46935</v>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>Fridge</t>
+          <t>Rack</t>
         </is>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>Pure, 2 fl oz</t>
         </is>
       </c>
       <c r="R8" s="7">
@@ -6141,12 +6145,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Cinnamon</t>
+          <t>Chocolate Chips</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Spice</t>
+          <t>Chocolate</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -6155,20 +6159,20 @@
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>100</v>
+        <v>340</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>4.5</v>
+        <v>4.49</v>
       </c>
       <c r="G9" s="24">
         <f>IF(E9=0,0,F9/E9)</f>
         <v/>
       </c>
       <c r="H9" s="8" t="n">
-        <v>45</v>
+        <v>1200</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>20</v>
+        <v>400</v>
       </c>
       <c r="J9" s="23">
         <f>H9*G9</f>
@@ -6180,26 +6184,26 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Spice Co</t>
+          <t>Nestlé Toll House</t>
         </is>
       </c>
       <c r="M9" s="25" t="n">
-        <v>45778</v>
+        <v>46246</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>100</v>
+        <v>680</v>
       </c>
       <c r="O9" s="25" t="n">
-        <v>46143</v>
+        <v>46600</v>
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Rack</t>
+          <t>Pantry B</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Ceylon</t>
+          <t>Semi-sweet, 12 oz</t>
         </is>
       </c>
       <c r="R9" s="8">
@@ -6213,12 +6217,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Sourdough Starter</t>
+          <t>Cream Cheese</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Starter</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -6227,20 +6231,20 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>500</v>
+        <v>226</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>0.5</v>
+        <v>2.29</v>
       </c>
       <c r="G10" s="21">
         <f>IF(E10=0,0,F10/E10)</f>
         <v/>
       </c>
       <c r="H10" s="7" t="n">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="J10" s="20">
         <f>H10*G10</f>
@@ -6252,16 +6256,18 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Homemade</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="M10" s="22" t="n">
-        <v>45857</v>
+        <v>46249</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>500</v>
-      </c>
-      <c r="O10" s="7" t="inlineStr"/>
+        <v>453</v>
+      </c>
+      <c r="O10" s="22" t="n">
+        <v>46275</v>
+      </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
           <t>Fridge</t>
@@ -6269,7 +6275,7 @@
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>Feed daily</t>
+          <t>8 oz — OUT OF STOCK</t>
         </is>
       </c>
       <c r="R10" s="7">
@@ -6283,34 +6289,34 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Heavy Cream</t>
+          <t>Cinnamon</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Spice</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>500</v>
+        <v>57</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>4.99</v>
+        <v>4.29</v>
       </c>
       <c r="G11" s="24">
         <f>IF(E11=0,0,F11/E11)</f>
         <v/>
       </c>
       <c r="H11" s="8" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="J11" s="23">
         <f>H11*G11</f>
@@ -6322,26 +6328,26 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>McCormick</t>
         </is>
       </c>
       <c r="M11" s="25" t="n">
-        <v>45855</v>
+        <v>46174</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>500</v>
+        <v>57</v>
       </c>
       <c r="O11" s="25" t="n">
-        <v>45863</v>
+        <v>46905</v>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Fridge</t>
+          <t>Rack</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Ground, 2 oz</t>
         </is>
       </c>
       <c r="R11" s="8">
@@ -6355,31 +6361,31 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Olive Oil</t>
+          <t>Sourdough Starter</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Oil</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
         <v>500</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>6.5</v>
+        <v>0.5</v>
       </c>
       <c r="G12" s="21">
         <f>IF(E12=0,0,F12/E12)</f>
         <v/>
       </c>
       <c r="H12" s="7" t="n">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>100</v>
@@ -6394,24 +6400,26 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>Olive Co</t>
+          <t>Homemade</t>
         </is>
       </c>
       <c r="M12" s="22" t="n">
-        <v>45839</v>
+        <v>46262</v>
       </c>
       <c r="N12" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="O12" s="22" t="n">
-        <v>46204</v>
-      </c>
+      <c r="O12" s="7" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>Pantry</t>
-        </is>
-      </c>
-      <c r="Q12" s="7" t="inlineStr"/>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>Feed weekly</t>
+        </is>
+      </c>
       <c r="R12" s="7">
         <f>IFERROR(VLOOKUP(D12,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
@@ -6423,34 +6431,34 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>All-Purpose Flour</t>
+          <t>Heavy Cream</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Flour</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>5000</v>
+        <v>473</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>5.5</v>
+        <v>3.99</v>
       </c>
       <c r="G13" s="24">
         <f>IF(E13=0,0,F13/E13)</f>
         <v/>
       </c>
       <c r="H13" s="8" t="n">
-        <v>3000</v>
+        <v>100</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="J13" s="23">
         <f>H13*G13</f>
@@ -6462,122 +6470,244 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>Bob's</t>
+          <t>Organic Valley</t>
         </is>
       </c>
       <c r="M13" s="25" t="n">
-        <v>45848</v>
+        <v>46259</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>5000</v>
+        <v>946</v>
       </c>
       <c r="O13" s="25" t="n">
-        <v>46023</v>
+        <v>46280</v>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Pantry A</t>
-        </is>
-      </c>
-      <c r="Q13" s="8" t="inlineStr"/>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>Pint — LOW STOCK</t>
+        </is>
+      </c>
       <c r="R13" s="8">
         <f>IFERROR(VLOOKUP(D13,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Olive Oil</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Oil</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="G14" s="21">
         <f>IF(E14=0,0,F14/E14)</f>
         <v/>
       </c>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7">
+      <c r="H14" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" s="20">
         <f>H14*G14</f>
         <v/>
       </c>
       <c r="K14" s="7">
-        <f>IF(H14="","",IF(H14=0,"OUT",IF(H14&lt;=I14,"LOW","OK")))</f>
-        <v/>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="7" t="n"/>
+        <f>IF(H14=0,"OUT",IF(H14&lt;=I14,"LOW","OK"))</f>
+        <v/>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>California Olive Ranch</t>
+        </is>
+      </c>
+      <c r="M14" s="22" t="n">
+        <v>46204</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="O14" s="22" t="n">
+        <v>46569</v>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pantry A</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>Extra virgin</t>
+        </is>
+      </c>
       <c r="R14" s="7">
-        <f>IF(D14="","",IFERROR(VLOOKUP(D14,'Unit Conversion'!A:B,2,FALSE),""))</f>
+        <f>IFERROR(VLOOKUP(D14,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Spice</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>1361</v>
+      </c>
+      <c r="F15" s="23" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="G15" s="24">
         <f>IF(E15=0,0,F15/E15)</f>
         <v/>
       </c>
-      <c r="H15" s="8" t="n"/>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8">
+      <c r="H15" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="J15" s="23">
         <f>H15*G15</f>
         <v/>
       </c>
       <c r="K15" s="8">
-        <f>IF(H15="","",IF(H15=0,"OUT",IF(H15&lt;=I15,"LOW","OK")))</f>
-        <v/>
-      </c>
-      <c r="L15" s="8" t="n"/>
-      <c r="M15" s="8" t="n"/>
-      <c r="N15" s="8" t="n"/>
-      <c r="O15" s="8" t="n"/>
-      <c r="P15" s="8" t="n"/>
-      <c r="Q15" s="8" t="n"/>
+        <f>IF(H15=0,"OUT",IF(H15&lt;=I15,"LOW","OK"))</f>
+        <v/>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Morton</t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="n">
+        <v>46218</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>1361</v>
+      </c>
+      <c r="O15" s="25" t="n">
+        <v>46935</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>Pantry A</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>Kosher, 3 lb</t>
+        </is>
+      </c>
       <c r="R15" s="8">
-        <f>IF(D15="","",IFERROR(VLOOKUP(D15,'Unit Conversion'!A:B,2,FALSE),""))</f>
+        <f>IFERROR(VLOOKUP(D15,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7">
+      <c r="A16" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>3785</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G16" s="21">
         <f>IF(E16=0,0,F16/E16)</f>
         <v/>
       </c>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7">
+      <c r="H16" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J16" s="20">
         <f>H16*G16</f>
         <v/>
       </c>
       <c r="K16" s="7">
-        <f>IF(H16="","",IF(H16=0,"OUT",IF(H16&lt;=I16,"LOW","OK")))</f>
-        <v/>
-      </c>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="n"/>
+        <f>IF(H16=0,"OUT",IF(H16&lt;=I16,"LOW","OK"))</f>
+        <v/>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Municipal</t>
+        </is>
+      </c>
+      <c r="M16" s="22" t="n">
+        <v>46262</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>3785</v>
+      </c>
+      <c r="O16" s="7" t="inlineStr"/>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Sink</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t>Tap water</t>
+        </is>
+      </c>
       <c r="R16" s="7">
-        <f>IF(D16="","",IFERROR(VLOOKUP(D16,'Unit Conversion'!A:B,2,FALSE),""))</f>
+        <f>IFERROR(VLOOKUP(D16,'Unit Conversion'!A:B,2,FALSE),"Weight")</f>
         <v/>
       </c>
     </row>
@@ -7966,7 +8096,7 @@
         <v>1.5</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I5" s="23">
         <f>G5*H5</f>
@@ -8051,7 +8181,7 @@
         <v>0.75</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I6" s="20">
         <f>G6*H6</f>
@@ -8136,7 +8266,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I7" s="23">
         <f>G7*H7</f>
@@ -8221,7 +8351,7 @@
         <v>0.5</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I8" s="20">
         <f>G8*H8</f>
@@ -8302,7 +8432,7 @@
         <v>1</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I9" s="23">
         <f>G9*H9</f>
@@ -30615,11 +30745,11 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>Cottage kitchen rent / shared kitchen</t>
+          <t>Shared commercial kitchen / home kitchen allocation</t>
         </is>
       </c>
       <c r="C5" s="35" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D5" s="33">
         <f>C5*12</f>
@@ -30644,7 +30774,7 @@
         </is>
       </c>
       <c r="C6" s="35" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="D6" s="33">
         <f>C6*12</f>
@@ -30665,11 +30795,11 @@
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>Liability + cottage food insurance</t>
+          <t>Cottage food liability + business policy</t>
         </is>
       </c>
       <c r="C7" s="35" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D7" s="33">
         <f>C7*12</f>
@@ -30690,7 +30820,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>Cottage food permit + business license</t>
+          <t>State cottage food permit + business license</t>
         </is>
       </c>
       <c r="C8" s="35" t="n">
@@ -30707,7 +30837,7 @@
       </c>
       <c r="F8" s="31" t="inlineStr">
         <is>
-          <t>$180/year</t>
+          <t>~$180/year</t>
         </is>
       </c>
     </row>
@@ -30719,11 +30849,11 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>Website + phone</t>
+          <t>Website + phone line</t>
         </is>
       </c>
       <c r="C9" s="35" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D9" s="33">
         <f>C9*12</f>
@@ -30744,11 +30874,11 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>Accounting + Sheets + Canva</t>
+          <t>Accounting + Google Workspace + Canva</t>
         </is>
       </c>
       <c r="C10" s="35" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D10" s="33">
         <f>C10*12</f>
@@ -30769,11 +30899,11 @@
       </c>
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>Instagram ads + flyers</t>
+          <t>Instagram/Facebook ads + flyers</t>
         </is>
       </c>
       <c r="C11" s="35" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D11" s="33">
         <f>C11*12</f>
@@ -30794,11 +30924,11 @@
       </c>
       <c r="B12" s="31" t="inlineStr">
         <is>
-          <t>Market gas + delivery</t>
+          <t>Farmers market gas + delivery</t>
         </is>
       </c>
       <c r="C12" s="35" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="D12" s="33">
         <f>C12*12</f>
@@ -30819,11 +30949,11 @@
       </c>
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>Storage bins + shelves</t>
+          <t>Bins, shelves, labels</t>
         </is>
       </c>
       <c r="C13" s="35" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="33">
         <f>C13*12</f>
@@ -30844,11 +30974,11 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>Supplies + cleaning</t>
+          <t>Sanitizer + cleaning supplies</t>
         </is>
       </c>
       <c r="C14" s="35" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D14" s="33">
         <f>C14*12</f>
@@ -30873,7 +31003,7 @@
         </is>
       </c>
       <c r="C15" s="35" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D15" s="33">
         <f>C15*12</f>
@@ -30894,11 +31024,11 @@
       </c>
       <c r="B16" s="31" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="C16" s="35" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D16" s="33">
         <f>C16*12</f>
@@ -31268,14 +31398,14 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>Stand Mixer KitchenAid 6qt</t>
+          <t>KitchenAid 6 qt stand mixer</t>
         </is>
       </c>
       <c r="C5" s="35" t="n">
-        <v>450</v>
+        <v>449.99</v>
       </c>
       <c r="D5" s="53" t="n">
-        <v>45667</v>
+        <v>46032</v>
       </c>
       <c r="E5" s="31" t="inlineStr">
         <is>
@@ -31299,18 +31429,18 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>Oven upgrade / Dutch oven</t>
+          <t>Dutch oven / oven upgrade</t>
         </is>
       </c>
       <c r="C6" s="35" t="n">
-        <v>300</v>
+        <v>349</v>
       </c>
       <c r="D6" s="53" t="n">
-        <v>45669</v>
+        <v>46034</v>
       </c>
       <c r="E6" s="31" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Sur La Table</t>
         </is>
       </c>
       <c r="F6" s="31" t="n">
@@ -31330,14 +31460,14 @@
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>Refrigerator extra</t>
+          <t>Extra refrigerator</t>
         </is>
       </c>
       <c r="C7" s="35" t="n">
-        <v>600</v>
+        <v>649</v>
       </c>
       <c r="D7" s="53" t="n">
-        <v>45672</v>
+        <v>46037</v>
       </c>
       <c r="E7" s="31" t="inlineStr">
         <is>
@@ -31361,14 +31491,14 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>Baking sheets, pans, bowls</t>
+          <t>Baking sheets, pans, mixing bowls</t>
         </is>
       </c>
       <c r="C8" s="35" t="n">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="D8" s="53" t="n">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="E8" s="31" t="inlineStr">
         <is>
@@ -31392,14 +31522,14 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>Packaging sealer + scale</t>
+          <t>Digital scale + packaging sealer</t>
         </is>
       </c>
       <c r="C9" s="35" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D9" s="53" t="n">
-        <v>45666</v>
+        <v>46031</v>
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
@@ -31423,14 +31553,14 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>Flour, sugar, butter initial stock</t>
+          <t>Flour, sugar, butter, eggs opening stock</t>
         </is>
       </c>
       <c r="C10" s="35" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="D10" s="53" t="n">
-        <v>45672</v>
+        <v>46037</v>
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
@@ -31458,18 +31588,18 @@
       </c>
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>Boxes, bags, labels, stickers initial</t>
+          <t>Boxes, bags, labels, stickers</t>
         </is>
       </c>
       <c r="C11" s="35" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="D11" s="53" t="n">
-        <v>45673</v>
+        <v>46038</v>
       </c>
       <c r="E11" s="31" t="inlineStr">
         <is>
-          <t>Pack Co</t>
+          <t>WebstaurantStore</t>
         </is>
       </c>
       <c r="F11" s="31" t="n">
@@ -31496,11 +31626,11 @@
         <v>200</v>
       </c>
       <c r="D12" s="53" t="n">
-        <v>45662</v>
+        <v>46027</v>
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>State / City</t>
         </is>
       </c>
       <c r="F12" s="31" t="n">
@@ -31512,7 +31642,7 @@
       </c>
       <c r="H12" s="31" t="inlineStr">
         <is>
-          <t>Annual but first year</t>
+          <t>First year</t>
         </is>
       </c>
     </row>
@@ -31531,11 +31661,11 @@
         <v>250</v>
       </c>
       <c r="D13" s="53" t="n">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="E13" s="31" t="inlineStr">
         <is>
-          <t>Fiverr + GoDaddy</t>
+          <t>Fiverr + Squarespace</t>
         </is>
       </c>
       <c r="F13" s="31" t="n">
@@ -31555,18 +31685,18 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>Initial flyers, banners, samples</t>
+          <t>Flyers, banners, samples</t>
         </is>
       </c>
       <c r="C14" s="35" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D14" s="53" t="n">
-        <v>45677</v>
+        <v>46042</v>
       </c>
       <c r="E14" s="31" t="inlineStr">
         <is>
-          <t>Local print</t>
+          <t>Local print shop</t>
         </is>
       </c>
       <c r="F14" s="31" t="n">
@@ -31586,14 +31716,14 @@
       </c>
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>Food safety manager certification</t>
+          <t>ServSafe Food Manager certification</t>
         </is>
       </c>
       <c r="C15" s="35" t="n">
         <v>150</v>
       </c>
       <c r="D15" s="53" t="n">
-        <v>45660</v>
+        <v>46025</v>
       </c>
       <c r="E15" s="31" t="inlineStr">
         <is>
@@ -31617,14 +31747,14 @@
       </c>
       <c r="B16" s="31" t="inlineStr">
         <is>
-          <t>Misc initial</t>
+          <t>Miscellaneous initial supplies</t>
         </is>
       </c>
       <c r="C16" s="35" t="n">
         <v>100</v>
       </c>
       <c r="D16" s="53" t="n">
-        <v>45682</v>
+        <v>46047</v>
       </c>
       <c r="E16" s="31" t="inlineStr"/>
       <c r="F16" s="31" t="n">

</xml_diff>

<commit_message>
Add Donation Stand version (free products + donations tracking), same layout
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cottage-bakery-spreadsheet/Cottage_Bakery_v4_ENHANCED.xlsx
+++ b/cottage-bakery-spreadsheet/Cottage_Bakery_v4_ENHANCED.xlsx
@@ -1991,11 +1991,11 @@
         </is>
       </c>
       <c r="B2" s="63" t="n">
-        <v>46254</v>
+        <v>46259</v>
       </c>
       <c r="C2" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D2" s="64" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B3" s="63" t="n">
-        <v>46248</v>
+        <v>46261</v>
       </c>
       <c r="C3" s="64" t="inlineStr">
         <is>
@@ -2103,11 +2103,11 @@
         </is>
       </c>
       <c r="B4" s="63" t="n">
-        <v>46260</v>
+        <v>46237</v>
       </c>
       <c r="C4" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D4" s="64" t="inlineStr">
@@ -2159,11 +2159,11 @@
         </is>
       </c>
       <c r="B5" s="63" t="n">
-        <v>46244</v>
+        <v>46236</v>
       </c>
       <c r="C5" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D5" s="64" t="inlineStr">
@@ -2215,11 +2215,11 @@
         </is>
       </c>
       <c r="B6" s="63" t="n">
-        <v>46251</v>
+        <v>46238</v>
       </c>
       <c r="C6" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D6" s="64" t="inlineStr">
@@ -2271,11 +2271,11 @@
         </is>
       </c>
       <c r="B7" s="63" t="n">
-        <v>46260</v>
+        <v>46245</v>
       </c>
       <c r="C7" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D7" s="64" t="inlineStr">
@@ -2327,11 +2327,11 @@
         </is>
       </c>
       <c r="B8" s="63" t="n">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="C8" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D8" s="64" t="inlineStr">
@@ -2383,11 +2383,11 @@
         </is>
       </c>
       <c r="B9" s="63" t="n">
-        <v>46260</v>
+        <v>46235</v>
       </c>
       <c r="C9" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D9" s="64" t="inlineStr">
@@ -2439,11 +2439,11 @@
         </is>
       </c>
       <c r="B10" s="63" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C10" s="64" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D10" s="64" t="inlineStr">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="B11" s="63" t="n">
-        <v>46253</v>
+        <v>46247</v>
       </c>
       <c r="C11" s="64" t="inlineStr">
         <is>
@@ -2551,11 +2551,11 @@
         </is>
       </c>
       <c r="B12" s="63" t="n">
-        <v>46243</v>
+        <v>46240</v>
       </c>
       <c r="C12" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D12" s="64" t="inlineStr">
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="B13" s="63" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="C13" s="64" t="inlineStr">
         <is>
@@ -2663,11 +2663,11 @@
         </is>
       </c>
       <c r="B14" s="63" t="n">
-        <v>46255</v>
+        <v>46241</v>
       </c>
       <c r="C14" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D14" s="64" t="inlineStr">
@@ -2719,11 +2719,11 @@
         </is>
       </c>
       <c r="B15" s="63" t="n">
-        <v>46252</v>
+        <v>46241</v>
       </c>
       <c r="C15" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D15" s="64" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="C16" s="64" t="inlineStr">
         <is>
-          <t>Emma Johnson</t>
+          <t>Liam Smith</t>
         </is>
       </c>
       <c r="D16" s="64" t="inlineStr">
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="B17" s="63" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="C17" s="64" t="inlineStr">
         <is>
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="B18" s="63" t="n">
-        <v>46261</v>
+        <v>46253</v>
       </c>
       <c r="C18" s="64" t="inlineStr">
         <is>
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="B19" s="63" t="n">
-        <v>46260</v>
+        <v>46237</v>
       </c>
       <c r="C19" s="64" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="B20" s="63" t="n">
-        <v>46235</v>
+        <v>46254</v>
       </c>
       <c r="C20" s="64" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="B21" s="63" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C21" s="64" t="inlineStr">
         <is>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="C2" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D2" s="31" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="C3" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D3" s="31" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="C7" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D7" s="31" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="C9" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D9" s="31" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="D10" s="31" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B2" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D2">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B4" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D4">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D5">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D7">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>Liam Smith</t>
+          <t>Emma Johnson</t>
         </is>
       </c>
       <c r="D10">

</xml_diff>